<commit_message>
update rka dari web
</commit_message>
<xml_diff>
--- a/data/rka.xlsx
+++ b/data/rka.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\76193\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A842523A-B681-4FB6-8DE4-C6B259D66125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{B926CE83-FEB6-4418-BD8D-37ADC92BA2FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
-    <sheet name="20260907 SAP ZFM01" sheetId="1" r:id="rId1"/>
+    <sheet name="20260911 SAP ZFM01" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1093" uniqueCount="131">
   <si>
     <t>Funds Center/Commitment Item</t>
   </si>
@@ -423,7 +423,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -560,7 +560,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -740,6 +740,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -901,8 +907,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1257,7 +1264,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H564"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1301,22 +1308,22 @@
         <v>8</v>
       </c>
       <c r="B2">
-        <v>109317656175</v>
+        <v>108940456175</v>
       </c>
       <c r="C2">
-        <v>109317656175</v>
+        <v>108940456175</v>
       </c>
       <c r="D2">
-        <v>99268647251</v>
+        <v>94287482435</v>
       </c>
       <c r="E2">
-        <v>8267348916</v>
+        <v>13248513732</v>
       </c>
       <c r="F2">
         <v>107535996167</v>
       </c>
       <c r="G2">
-        <v>1781660008</v>
+        <v>1404460008</v>
       </c>
       <c r="H2" t="s">
         <v>9</v>
@@ -1463,10 +1470,10 @@
         <v>3726972261</v>
       </c>
       <c r="D8">
-        <v>3622271715</v>
+        <v>3398631820</v>
       </c>
       <c r="E8">
-        <v>77164840</v>
+        <v>300804735</v>
       </c>
       <c r="F8">
         <v>3699436555</v>
@@ -1489,10 +1496,10 @@
         <v>62772333130</v>
       </c>
       <c r="D9">
-        <v>54589308663</v>
+        <v>37626079655</v>
       </c>
       <c r="E9">
-        <v>8154071362</v>
+        <v>25117300370</v>
       </c>
       <c r="F9">
         <v>62743380025</v>
@@ -1509,22 +1516,22 @@
         <v>17</v>
       </c>
       <c r="B10">
-        <v>579317296</v>
+        <v>490324430</v>
       </c>
       <c r="C10">
-        <v>579317296</v>
+        <v>490324430</v>
       </c>
       <c r="D10">
-        <v>197598375</v>
+        <v>148038375</v>
       </c>
       <c r="E10">
-        <v>192718055</v>
+        <v>242278055</v>
       </c>
       <c r="F10">
         <v>390316430</v>
       </c>
       <c r="G10">
-        <v>189000866</v>
+        <v>100008000</v>
       </c>
       <c r="H10" t="s">
         <v>9</v>
@@ -1691,7 +1698,7 @@
         <v>24</v>
       </c>
       <c r="B17">
-        <v>1600000000</v>
+        <v>1200000000</v>
       </c>
       <c r="C17">
         <v>1200000000</v>
@@ -1708,8 +1715,8 @@
       <c r="G17">
         <v>1015199000</v>
       </c>
-      <c r="H17">
-        <v>400000000</v>
+      <c r="H17" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
@@ -1717,10 +1724,10 @@
         <v>25</v>
       </c>
       <c r="B18">
-        <v>454442400</v>
+        <v>391942400</v>
       </c>
       <c r="C18">
-        <v>329442400</v>
+        <v>391942400</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -1732,10 +1739,10 @@
         <v>20986164</v>
       </c>
       <c r="G18">
-        <v>308456236</v>
-      </c>
-      <c r="H18">
-        <v>125000000</v>
+        <v>370956236</v>
+      </c>
+      <c r="H18" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
@@ -1743,10 +1750,10 @@
         <v>26</v>
       </c>
       <c r="B19">
-        <v>4500000000</v>
+        <v>3894602130</v>
       </c>
       <c r="C19">
-        <v>4500000000</v>
+        <v>3894602130</v>
       </c>
       <c r="D19">
         <v>346244860</v>
@@ -1758,7 +1765,7 @@
         <v>2910182489</v>
       </c>
       <c r="G19">
-        <v>1589817511</v>
+        <v>984419641</v>
       </c>
       <c r="H19" t="s">
         <v>9</v>
@@ -1769,10 +1776,10 @@
         <v>27</v>
       </c>
       <c r="B20">
-        <v>1483013800</v>
+        <v>1000698000</v>
       </c>
       <c r="C20">
-        <v>1108013800</v>
+        <v>1000698000</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -1784,10 +1791,10 @@
         <v>406948000</v>
       </c>
       <c r="G20">
-        <v>701065800</v>
-      </c>
-      <c r="H20">
-        <v>375000000</v>
+        <v>593750000</v>
+      </c>
+      <c r="H20" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
@@ -1795,25 +1802,25 @@
         <v>28</v>
       </c>
       <c r="B21">
-        <v>702885000</v>
+        <v>406635000</v>
       </c>
       <c r="C21">
-        <v>510385000</v>
+        <v>406635000</v>
       </c>
       <c r="D21">
-        <v>75773600</v>
+        <v>77481217</v>
       </c>
       <c r="E21">
-        <v>84557037</v>
+        <v>89696662</v>
       </c>
       <c r="F21">
-        <v>160330637</v>
+        <v>167177879</v>
       </c>
       <c r="G21">
-        <v>350054363</v>
-      </c>
-      <c r="H21">
-        <v>192500000</v>
+        <v>239457121</v>
+      </c>
+      <c r="H21" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
@@ -1821,10 +1828,10 @@
         <v>29</v>
       </c>
       <c r="B22">
-        <v>156000000</v>
+        <v>146000000</v>
       </c>
       <c r="C22">
-        <v>156000000</v>
+        <v>146000000</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -1836,7 +1843,7 @@
         <v>103000000</v>
       </c>
       <c r="G22">
-        <v>53000000</v>
+        <v>43000000</v>
       </c>
       <c r="H22" t="s">
         <v>9</v>
@@ -1847,25 +1854,25 @@
         <v>30</v>
       </c>
       <c r="B23">
-        <v>747597314</v>
+        <v>685097314</v>
       </c>
       <c r="C23">
-        <v>622597314</v>
+        <v>685097314</v>
       </c>
       <c r="D23">
-        <v>507783920</v>
+        <v>551635520</v>
       </c>
       <c r="E23">
         <v>114645294</v>
       </c>
       <c r="F23">
-        <v>622429214</v>
+        <v>666280814</v>
       </c>
       <c r="G23">
-        <v>168100</v>
-      </c>
-      <c r="H23">
-        <v>125000000</v>
+        <v>18816500</v>
+      </c>
+      <c r="H23" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
@@ -1873,7 +1880,7 @@
         <v>31</v>
       </c>
       <c r="B24">
-        <v>800000000</v>
+        <v>600000000</v>
       </c>
       <c r="C24">
         <v>600000000</v>
@@ -1890,8 +1897,8 @@
       <c r="G24">
         <v>353609968</v>
       </c>
-      <c r="H24">
-        <v>200000000</v>
+      <c r="H24" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
@@ -1899,25 +1906,25 @@
         <v>32</v>
       </c>
       <c r="B25">
-        <v>2312674754</v>
+        <v>1691277133</v>
       </c>
       <c r="C25">
-        <v>1687674754</v>
+        <v>1691277133</v>
       </c>
       <c r="D25">
         <v>215556103</v>
       </c>
       <c r="E25">
-        <v>1066286941</v>
+        <v>1088880691</v>
       </c>
       <c r="F25">
-        <v>1281843044</v>
+        <v>1304436794</v>
       </c>
       <c r="G25">
-        <v>405831710</v>
-      </c>
-      <c r="H25">
-        <v>625000000</v>
+        <v>386840339</v>
+      </c>
+      <c r="H25" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
@@ -1925,10 +1932,10 @@
         <v>33</v>
       </c>
       <c r="B26">
-        <v>220000000</v>
+        <v>128132588</v>
       </c>
       <c r="C26">
-        <v>220000000</v>
+        <v>128132588</v>
       </c>
       <c r="D26">
         <v>0</v>
@@ -1940,7 +1947,7 @@
         <v>28132588</v>
       </c>
       <c r="G26">
-        <v>191867412</v>
+        <v>100000000</v>
       </c>
       <c r="H26" t="s">
         <v>9</v>
@@ -1986,13 +1993,13 @@
         <v>0</v>
       </c>
       <c r="E28">
-        <v>2833990776</v>
+        <v>2834764214</v>
       </c>
       <c r="F28">
-        <v>2833990776</v>
+        <v>2834764214</v>
       </c>
       <c r="G28">
-        <v>622623428</v>
+        <v>621849990</v>
       </c>
       <c r="H28" t="s">
         <v>9</v>
@@ -2038,13 +2045,13 @@
         <v>0</v>
       </c>
       <c r="E30">
-        <v>3661908187</v>
+        <v>3669312187</v>
       </c>
       <c r="F30">
-        <v>3661908187</v>
+        <v>3669312187</v>
       </c>
       <c r="G30">
-        <v>416361848</v>
+        <v>408957848</v>
       </c>
       <c r="H30" t="s">
         <v>9</v>
@@ -2142,13 +2149,13 @@
         <v>0</v>
       </c>
       <c r="E34">
-        <v>10058200960</v>
+        <v>10062254960</v>
       </c>
       <c r="F34">
-        <v>10058200960</v>
+        <v>10062254960</v>
       </c>
       <c r="G34">
-        <v>3911865086</v>
+        <v>3907811086</v>
       </c>
       <c r="H34" t="s">
         <v>9</v>
@@ -2263,10 +2270,10 @@
         <v>46</v>
       </c>
       <c r="B39">
-        <v>752402686</v>
+        <v>274300566</v>
       </c>
       <c r="C39">
-        <v>502402686</v>
+        <v>274300566</v>
       </c>
       <c r="D39">
         <v>0</v>
@@ -2278,10 +2285,10 @@
         <v>8807378</v>
       </c>
       <c r="G39">
-        <v>493595308</v>
-      </c>
-      <c r="H39">
-        <v>250000000</v>
+        <v>265493188</v>
+      </c>
+      <c r="H39" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
@@ -2289,10 +2296,10 @@
         <v>47</v>
       </c>
       <c r="B40">
-        <v>500000000</v>
+        <v>437500000</v>
       </c>
       <c r="C40">
-        <v>375000000</v>
+        <v>437500000</v>
       </c>
       <c r="D40">
         <v>0</v>
@@ -2304,10 +2311,10 @@
         <v>15794000</v>
       </c>
       <c r="G40">
-        <v>359206000</v>
-      </c>
-      <c r="H40">
-        <v>125000000</v>
+        <v>421706000</v>
+      </c>
+      <c r="H40" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
@@ -2341,25 +2348,25 @@
         <v>49</v>
       </c>
       <c r="B42">
-        <v>350773419540</v>
+        <v>346934395851</v>
       </c>
       <c r="C42">
-        <v>348355919540</v>
+        <v>346934395851</v>
       </c>
       <c r="D42">
-        <v>237558913890</v>
+        <v>215386879388</v>
       </c>
       <c r="E42">
-        <v>94119402504</v>
+        <v>116376961036</v>
       </c>
       <c r="F42">
-        <v>331678316394</v>
+        <v>331763840424</v>
       </c>
       <c r="G42">
-        <v>16677603146</v>
-      </c>
-      <c r="H42">
-        <v>2417500000</v>
+        <v>15170555427</v>
+      </c>
+      <c r="H42" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
@@ -2373,16 +2380,16 @@
         <v>26681487101</v>
       </c>
       <c r="D43">
-        <v>17366902401</v>
+        <v>17343493202</v>
       </c>
       <c r="E43">
         <v>9295238000</v>
       </c>
       <c r="F43">
-        <v>26662140401</v>
+        <v>26638731202</v>
       </c>
       <c r="G43">
-        <v>19346700</v>
+        <v>42755899</v>
       </c>
       <c r="H43" t="s">
         <v>9</v>
@@ -2607,16 +2614,16 @@
         <v>400000000</v>
       </c>
       <c r="D52">
-        <v>399980984</v>
+        <v>391600000</v>
       </c>
       <c r="E52">
         <v>0</v>
       </c>
       <c r="F52">
-        <v>399980984</v>
+        <v>391600000</v>
       </c>
       <c r="G52">
-        <v>19016</v>
+        <v>8400000</v>
       </c>
       <c r="H52" t="s">
         <v>9</v>
@@ -2659,16 +2666,16 @@
         <v>6000000000</v>
       </c>
       <c r="D54">
-        <v>5252888358</v>
+        <v>5229810269</v>
       </c>
       <c r="E54">
         <v>541614545</v>
       </c>
       <c r="F54">
-        <v>5794502903</v>
+        <v>5771424814</v>
       </c>
       <c r="G54">
-        <v>205497097</v>
+        <v>228575186</v>
       </c>
       <c r="H54" t="s">
         <v>9</v>
@@ -2685,16 +2692,16 @@
         <v>4260000000</v>
       </c>
       <c r="D55">
-        <v>1541830234</v>
+        <v>1178332074</v>
       </c>
       <c r="E55">
-        <v>2204642978</v>
+        <v>2608784178</v>
       </c>
       <c r="F55">
-        <v>3746473212</v>
+        <v>3787116252</v>
       </c>
       <c r="G55">
-        <v>513526788</v>
+        <v>472883748</v>
       </c>
       <c r="H55" t="s">
         <v>9</v>
@@ -2763,10 +2770,10 @@
         <v>250000000</v>
       </c>
       <c r="D58">
-        <v>75748702</v>
+        <v>0</v>
       </c>
       <c r="E58">
-        <v>73804960</v>
+        <v>149553662</v>
       </c>
       <c r="F58">
         <v>149553662</v>
@@ -2815,16 +2822,16 @@
         <v>2620000000</v>
       </c>
       <c r="D60">
-        <v>704306959</v>
+        <v>652442541</v>
       </c>
       <c r="E60">
-        <v>762786867</v>
+        <v>815038867</v>
       </c>
       <c r="F60">
-        <v>1467093826</v>
+        <v>1467481408</v>
       </c>
       <c r="G60">
-        <v>1152906174</v>
+        <v>1152518592</v>
       </c>
       <c r="H60" t="s">
         <v>9</v>
@@ -2893,16 +2900,16 @@
         <v>2500000000</v>
       </c>
       <c r="D63">
-        <v>2007946000</v>
+        <v>1948112000</v>
       </c>
       <c r="E63">
-        <v>333260100</v>
+        <v>383110100</v>
       </c>
       <c r="F63">
-        <v>2341206100</v>
+        <v>2331222100</v>
       </c>
       <c r="G63">
-        <v>158793900</v>
+        <v>168777900</v>
       </c>
       <c r="H63" t="s">
         <v>9</v>
@@ -2945,16 +2952,16 @@
         <v>180000150</v>
       </c>
       <c r="D65">
-        <v>9176000</v>
+        <v>31856000</v>
       </c>
       <c r="E65">
         <v>139677600</v>
       </c>
       <c r="F65">
-        <v>148853600</v>
+        <v>171533600</v>
       </c>
       <c r="G65">
-        <v>31146550</v>
+        <v>8466550</v>
       </c>
       <c r="H65" t="s">
         <v>9</v>
@@ -3130,13 +3137,13 @@
         <v>46676000</v>
       </c>
       <c r="E72">
-        <v>253203000</v>
+        <v>258971750</v>
       </c>
       <c r="F72">
-        <v>299879000</v>
+        <v>305647750</v>
       </c>
       <c r="G72">
-        <v>54346000</v>
+        <v>48577250</v>
       </c>
       <c r="H72">
         <v>118075000</v>
@@ -3208,13 +3215,13 @@
         <v>0</v>
       </c>
       <c r="E75">
-        <v>16580866780</v>
+        <v>16581026155</v>
       </c>
       <c r="F75">
-        <v>16580866780</v>
+        <v>16581026155</v>
       </c>
       <c r="G75">
-        <v>6350740449</v>
+        <v>6350581074</v>
       </c>
       <c r="H75" t="s">
         <v>9</v>
@@ -3257,10 +3264,10 @@
         <v>20967421530</v>
       </c>
       <c r="D77">
-        <v>62448139</v>
+        <v>9566218</v>
       </c>
       <c r="E77">
-        <v>17994131226</v>
+        <v>18047013147</v>
       </c>
       <c r="F77">
         <v>18056579365</v>
@@ -3361,10 +3368,10 @@
         <v>1937118528</v>
       </c>
       <c r="D81">
-        <v>1099501</v>
+        <v>165657</v>
       </c>
       <c r="E81">
-        <v>1889267075</v>
+        <v>1890200919</v>
       </c>
       <c r="F81">
         <v>1890366576</v>
@@ -3439,16 +3446,16 @@
         <v>110881210191</v>
       </c>
       <c r="D84">
-        <v>36852239634</v>
+        <v>36215290317</v>
       </c>
       <c r="E84">
-        <v>57297214607</v>
+        <v>57938950399</v>
       </c>
       <c r="F84">
-        <v>94149454241</v>
+        <v>94154240716</v>
       </c>
       <c r="G84">
-        <v>16731755950</v>
+        <v>16726969475</v>
       </c>
       <c r="H84">
         <v>671501500</v>
@@ -3569,16 +3576,16 @@
         <v>30639775739</v>
       </c>
       <c r="D89">
-        <v>14015063637</v>
+        <v>16314020110</v>
       </c>
       <c r="E89">
         <v>11956954821</v>
       </c>
       <c r="F89">
-        <v>25972018458</v>
+        <v>28270974931</v>
       </c>
       <c r="G89">
-        <v>4667757281</v>
+        <v>2368800808</v>
       </c>
       <c r="H89" t="s">
         <v>9</v>
@@ -3699,16 +3706,16 @@
         <v>2796520000</v>
       </c>
       <c r="D94">
-        <v>761898804</v>
+        <v>768155804</v>
       </c>
       <c r="E94">
         <v>2028357617</v>
       </c>
       <c r="F94">
-        <v>2790256421</v>
+        <v>2796513421</v>
       </c>
       <c r="G94">
-        <v>6263579</v>
+        <v>6579</v>
       </c>
       <c r="H94" t="s">
         <v>9</v>
@@ -3803,16 +3810,16 @@
         <v>289155000</v>
       </c>
       <c r="D98">
-        <v>20359000</v>
+        <v>38159000</v>
       </c>
       <c r="E98">
         <v>57100000</v>
       </c>
       <c r="F98">
-        <v>77459000</v>
+        <v>95259000</v>
       </c>
       <c r="G98">
-        <v>211696000</v>
+        <v>193896000</v>
       </c>
       <c r="H98" t="s">
         <v>9</v>
@@ -3829,16 +3836,16 @@
         <v>360000000</v>
       </c>
       <c r="D99">
-        <v>105051976</v>
+        <v>141522576</v>
       </c>
       <c r="E99">
         <v>204218000</v>
       </c>
       <c r="F99">
-        <v>309269976</v>
+        <v>345740576</v>
       </c>
       <c r="G99">
-        <v>50730024</v>
+        <v>14259424</v>
       </c>
       <c r="H99" t="s">
         <v>9</v>
@@ -3855,16 +3862,16 @@
         <v>1710494400</v>
       </c>
       <c r="D100">
-        <v>598275580</v>
+        <v>484281260</v>
       </c>
       <c r="E100">
         <v>1099212506</v>
       </c>
       <c r="F100">
-        <v>1697488086</v>
+        <v>1583493766</v>
       </c>
       <c r="G100">
-        <v>13006314</v>
+        <v>127000634</v>
       </c>
       <c r="H100" t="s">
         <v>9</v>
@@ -3907,16 +3914,16 @@
         <v>394475000</v>
       </c>
       <c r="D102">
-        <v>119148000</v>
+        <v>70510900</v>
       </c>
       <c r="E102">
         <v>45427850</v>
       </c>
       <c r="F102">
-        <v>164575850</v>
+        <v>115938750</v>
       </c>
       <c r="G102">
-        <v>229899150</v>
+        <v>278536250</v>
       </c>
       <c r="H102">
         <v>139825000</v>
@@ -3933,16 +3940,16 @@
         <v>255960000</v>
       </c>
       <c r="D103">
-        <v>65004150</v>
+        <v>60960230</v>
       </c>
       <c r="E103">
         <v>174999400</v>
       </c>
       <c r="F103">
-        <v>240003550</v>
+        <v>235959630</v>
       </c>
       <c r="G103">
-        <v>15956450</v>
+        <v>20000370</v>
       </c>
       <c r="H103">
         <v>85320000</v>
@@ -3985,16 +3992,16 @@
         <v>291600000</v>
       </c>
       <c r="D105">
-        <v>220821700</v>
+        <v>243281700</v>
       </c>
       <c r="E105">
         <v>28079000</v>
       </c>
       <c r="F105">
-        <v>248900700</v>
+        <v>271360700</v>
       </c>
       <c r="G105">
-        <v>42699300</v>
+        <v>20239300</v>
       </c>
       <c r="H105">
         <v>97200000</v>
@@ -4040,13 +4047,13 @@
         <v>0</v>
       </c>
       <c r="E107">
-        <v>291366068</v>
+        <v>292803568</v>
       </c>
       <c r="F107">
-        <v>291366068</v>
+        <v>292803568</v>
       </c>
       <c r="G107">
-        <v>3691432</v>
+        <v>2253932</v>
       </c>
       <c r="H107">
         <v>98352500</v>
@@ -4170,13 +4177,13 @@
         <v>0</v>
       </c>
       <c r="E112">
-        <v>11992041949</v>
+        <v>11992098199</v>
       </c>
       <c r="F112">
-        <v>11992041949</v>
+        <v>11992098199</v>
       </c>
       <c r="G112">
-        <v>4231602904</v>
+        <v>4231546654</v>
       </c>
       <c r="H112" t="s">
         <v>9</v>
@@ -4219,10 +4226,10 @@
         <v>14498179948</v>
       </c>
       <c r="D114">
-        <v>54284729</v>
+        <v>9868545</v>
       </c>
       <c r="E114">
-        <v>13036981539</v>
+        <v>13081397723</v>
       </c>
       <c r="F114">
         <v>13091266268</v>
@@ -4323,10 +4330,10 @@
         <v>1928660874</v>
       </c>
       <c r="D118">
-        <v>194430</v>
+        <v>0</v>
       </c>
       <c r="E118">
-        <v>1493780716</v>
+        <v>1493975146</v>
       </c>
       <c r="F118">
         <v>1493975146</v>
@@ -4401,16 +4408,16 @@
         <v>81693644736</v>
       </c>
       <c r="D121">
-        <v>18868718909</v>
+        <v>21039377028</v>
       </c>
       <c r="E121">
-        <v>50086023534</v>
+        <v>50132127898</v>
       </c>
       <c r="F121">
-        <v>68954742443</v>
+        <v>71171504926</v>
       </c>
       <c r="G121">
-        <v>12738902293</v>
+        <v>10522139810</v>
       </c>
       <c r="H121">
         <v>475697500</v>
@@ -4453,16 +4460,16 @@
         <v>1494332364</v>
       </c>
       <c r="D123">
-        <v>491000000</v>
+        <v>985946819</v>
       </c>
       <c r="E123">
         <v>127583711</v>
       </c>
       <c r="F123">
-        <v>618583711</v>
+        <v>1113530530</v>
       </c>
       <c r="G123">
-        <v>875748653</v>
+        <v>380801834</v>
       </c>
       <c r="H123" t="s">
         <v>9</v>
@@ -4531,16 +4538,16 @@
         <v>1200699000</v>
       </c>
       <c r="D126">
-        <v>668247328</v>
+        <v>662998053</v>
       </c>
       <c r="E126">
         <v>81220975</v>
       </c>
       <c r="F126">
-        <v>749468303</v>
+        <v>744219028</v>
       </c>
       <c r="G126">
-        <v>451230697</v>
+        <v>456479972</v>
       </c>
       <c r="H126" t="s">
         <v>9</v>
@@ -4557,10 +4564,10 @@
         <v>818532000</v>
       </c>
       <c r="D127">
-        <v>494768983</v>
+        <v>333965683</v>
       </c>
       <c r="E127">
-        <v>287074500</v>
+        <v>447877800</v>
       </c>
       <c r="F127">
         <v>781843483</v>
@@ -4583,16 +4590,16 @@
         <v>4824864000</v>
       </c>
       <c r="D128">
-        <v>0</v>
+        <v>1685220</v>
       </c>
       <c r="E128">
         <v>4612652831</v>
       </c>
       <c r="F128">
-        <v>4612652831</v>
+        <v>4614338051</v>
       </c>
       <c r="G128">
-        <v>212211169</v>
+        <v>210525949</v>
       </c>
       <c r="H128" t="s">
         <v>9</v>
@@ -4609,16 +4616,16 @@
         <v>1665000000</v>
       </c>
       <c r="D129">
-        <v>144401157</v>
+        <v>212643952</v>
       </c>
       <c r="E129">
         <v>713065052</v>
       </c>
       <c r="F129">
-        <v>857466209</v>
+        <v>925709004</v>
       </c>
       <c r="G129">
-        <v>807533791</v>
+        <v>739290996</v>
       </c>
       <c r="H129" t="s">
         <v>9</v>
@@ -4788,7 +4795,7 @@
         <v>705000000</v>
       </c>
       <c r="C136">
-        <v>528750000</v>
+        <v>593920000</v>
       </c>
       <c r="D136">
         <v>0</v>
@@ -4800,10 +4807,10 @@
         <v>491500000</v>
       </c>
       <c r="G136">
-        <v>37250000</v>
+        <v>102420000</v>
       </c>
       <c r="H136">
-        <v>176250000</v>
+        <v>111080000</v>
       </c>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.3">
@@ -4817,16 +4824,16 @@
         <v>118875000</v>
       </c>
       <c r="D137">
-        <v>3172500</v>
+        <v>14682500</v>
       </c>
       <c r="E137">
         <v>62015400</v>
       </c>
       <c r="F137">
-        <v>65187900</v>
+        <v>76697900</v>
       </c>
       <c r="G137">
-        <v>53687100</v>
+        <v>42177100</v>
       </c>
       <c r="H137" t="s">
         <v>9</v>
@@ -4866,22 +4873,22 @@
         <v>100000000</v>
       </c>
       <c r="C139">
-        <v>75000000</v>
+        <v>100000000</v>
       </c>
       <c r="D139">
-        <v>0</v>
+        <v>7999750</v>
       </c>
       <c r="E139">
         <v>74403889</v>
       </c>
       <c r="F139">
-        <v>74403889</v>
+        <v>82403639</v>
       </c>
       <c r="G139">
-        <v>596111</v>
-      </c>
-      <c r="H139">
-        <v>25000000</v>
+        <v>17596361</v>
+      </c>
+      <c r="H139" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.3">
@@ -4892,22 +4899,22 @@
         <v>354600000</v>
       </c>
       <c r="C140">
-        <v>265950000</v>
+        <v>354600000</v>
       </c>
       <c r="D140">
-        <v>11555000</v>
+        <v>4357100</v>
       </c>
       <c r="E140">
-        <v>209966600</v>
+        <v>220966600</v>
       </c>
       <c r="F140">
-        <v>221521600</v>
+        <v>225323700</v>
       </c>
       <c r="G140">
-        <v>44428400</v>
-      </c>
-      <c r="H140">
-        <v>88650000</v>
+        <v>129276300</v>
+      </c>
+      <c r="H140" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="141" spans="1:8" x14ac:dyDescent="0.3">
@@ -4944,7 +4951,7 @@
         <v>271400000</v>
       </c>
       <c r="C142">
-        <v>203550000</v>
+        <v>271400000</v>
       </c>
       <c r="D142">
         <v>2380000</v>
@@ -4956,10 +4963,10 @@
         <v>179583982</v>
       </c>
       <c r="G142">
-        <v>23966018</v>
-      </c>
-      <c r="H142">
-        <v>67850000</v>
+        <v>91816018</v>
+      </c>
+      <c r="H142" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.3">
@@ -4970,22 +4977,22 @@
         <v>213320000</v>
       </c>
       <c r="C143">
-        <v>159990000</v>
+        <v>213320000</v>
       </c>
       <c r="D143">
         <v>0</v>
       </c>
       <c r="E143">
-        <v>152110750</v>
+        <v>152660750</v>
       </c>
       <c r="F143">
-        <v>152110750</v>
+        <v>152660750</v>
       </c>
       <c r="G143">
-        <v>7879250</v>
-      </c>
-      <c r="H143">
-        <v>53330000</v>
+        <v>60659250</v>
+      </c>
+      <c r="H143" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.3">
@@ -5054,13 +5061,13 @@
         <v>0</v>
       </c>
       <c r="E146">
-        <v>7120196100</v>
+        <v>7120218600</v>
       </c>
       <c r="F146">
-        <v>7120196100</v>
+        <v>7120218600</v>
       </c>
       <c r="G146">
-        <v>2828897983</v>
+        <v>2828875483</v>
       </c>
       <c r="H146" t="s">
         <v>9</v>
@@ -5106,13 +5113,13 @@
         <v>0</v>
       </c>
       <c r="E148">
-        <v>8371186419</v>
+        <v>8399118521</v>
       </c>
       <c r="F148">
-        <v>8371186419</v>
+        <v>8399118521</v>
       </c>
       <c r="G148">
-        <v>1398663472</v>
+        <v>1370731370</v>
       </c>
       <c r="H148" t="s">
         <v>9</v>
@@ -5210,13 +5217,13 @@
         <v>0</v>
       </c>
       <c r="E152">
-        <v>1071715901</v>
+        <v>1073128014</v>
       </c>
       <c r="F152">
-        <v>1071715901</v>
+        <v>1073128014</v>
       </c>
       <c r="G152">
-        <v>258601638</v>
+        <v>257189525</v>
       </c>
       <c r="H152" t="s">
         <v>9</v>
@@ -5282,22 +5289,22 @@
         <v>52584136175</v>
       </c>
       <c r="C155">
-        <v>52173056175</v>
+        <v>52473056175</v>
       </c>
       <c r="D155">
-        <v>9723132060</v>
+        <v>10134266169</v>
       </c>
       <c r="E155">
-        <v>32526968870</v>
+        <v>32728688885</v>
       </c>
       <c r="F155">
-        <v>42250100930</v>
+        <v>42862955054</v>
       </c>
       <c r="G155">
-        <v>9922955245</v>
+        <v>9610101121</v>
       </c>
       <c r="H155">
-        <v>411080000</v>
+        <v>111080000</v>
       </c>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.3">
@@ -5597,16 +5604,16 @@
         <v>500000000</v>
       </c>
       <c r="D167">
-        <v>54664725</v>
+        <v>0</v>
       </c>
       <c r="E167">
         <v>185788488</v>
       </c>
       <c r="F167">
-        <v>240453213</v>
+        <v>185788488</v>
       </c>
       <c r="G167">
-        <v>259546787</v>
+        <v>314211512</v>
       </c>
       <c r="H167" t="s">
         <v>9</v>
@@ -5649,10 +5656,10 @@
         <v>867942000</v>
       </c>
       <c r="D169">
-        <v>642565410</v>
+        <v>235899000</v>
       </c>
       <c r="E169">
-        <v>0</v>
+        <v>406666410</v>
       </c>
       <c r="F169">
         <v>642565410</v>
@@ -5675,10 +5682,10 @@
         <v>187500000</v>
       </c>
       <c r="D170">
+        <v>0</v>
+      </c>
+      <c r="E170">
         <v>142100000</v>
-      </c>
-      <c r="E170">
-        <v>0</v>
       </c>
       <c r="F170">
         <v>142100000</v>
@@ -5805,16 +5812,16 @@
         <v>595150000</v>
       </c>
       <c r="D175">
-        <v>73181400</v>
+        <v>70019500</v>
       </c>
       <c r="E175">
         <v>451500394</v>
       </c>
       <c r="F175">
-        <v>524681794</v>
+        <v>521519894</v>
       </c>
       <c r="G175">
-        <v>70468206</v>
+        <v>73630106</v>
       </c>
       <c r="H175">
         <v>136250000</v>
@@ -5857,16 +5864,16 @@
         <v>253250000</v>
       </c>
       <c r="D177">
-        <v>49900000</v>
+        <v>104564725</v>
       </c>
       <c r="E177">
         <v>104678200</v>
       </c>
       <c r="F177">
-        <v>154578200</v>
+        <v>209242925</v>
       </c>
       <c r="G177">
-        <v>98671800</v>
+        <v>44007075</v>
       </c>
       <c r="H177">
         <v>146550000</v>
@@ -5912,13 +5919,13 @@
         <v>0</v>
       </c>
       <c r="E179">
-        <v>115634250</v>
+        <v>127765250</v>
       </c>
       <c r="F179">
-        <v>115634250</v>
+        <v>127765250</v>
       </c>
       <c r="G179">
-        <v>46667250</v>
+        <v>34536250</v>
       </c>
       <c r="H179">
         <v>54100500</v>
@@ -5964,13 +5971,13 @@
         <v>0</v>
       </c>
       <c r="E181">
-        <v>5304783338</v>
+        <v>5305580738</v>
       </c>
       <c r="F181">
-        <v>5304783338</v>
+        <v>5305580738</v>
       </c>
       <c r="G181">
-        <v>2199940040</v>
+        <v>2199142640</v>
       </c>
       <c r="H181" t="s">
         <v>9</v>
@@ -6169,16 +6176,16 @@
         <v>46375593027</v>
       </c>
       <c r="D189">
-        <v>10089378160</v>
+        <v>9537449850</v>
       </c>
       <c r="E189">
-        <v>28698856885</v>
+        <v>29260551695</v>
       </c>
       <c r="F189">
-        <v>38788235045</v>
+        <v>38798001545</v>
       </c>
       <c r="G189">
-        <v>7587357982</v>
+        <v>7577591482</v>
       </c>
       <c r="H189">
         <v>449400500</v>
@@ -6481,10 +6488,10 @@
         <v>1862650000</v>
       </c>
       <c r="D201">
-        <v>345529067</v>
+        <v>300009067</v>
       </c>
       <c r="E201">
-        <v>1370639706</v>
+        <v>1416159706</v>
       </c>
       <c r="F201">
         <v>1716168773</v>
@@ -6585,16 +6592,16 @@
         <v>4350172680</v>
       </c>
       <c r="D205">
-        <v>3109885000</v>
+        <v>2986575000</v>
       </c>
       <c r="E205">
         <v>1236281200</v>
       </c>
       <c r="F205">
-        <v>4346166200</v>
+        <v>4222856200</v>
       </c>
       <c r="G205">
-        <v>4006480</v>
+        <v>127316480</v>
       </c>
       <c r="H205" t="s">
         <v>9</v>
@@ -6611,16 +6618,16 @@
         <v>40000000</v>
       </c>
       <c r="D206">
-        <v>0</v>
+        <v>7640000</v>
       </c>
       <c r="E206">
         <v>13010000</v>
       </c>
       <c r="F206">
-        <v>13010000</v>
+        <v>20650000</v>
       </c>
       <c r="G206">
-        <v>26990000</v>
+        <v>19350000</v>
       </c>
       <c r="H206" t="s">
         <v>9</v>
@@ -6761,25 +6768,25 @@
         <v>27</v>
       </c>
       <c r="B212">
-        <v>130000000</v>
+        <v>113750000</v>
       </c>
       <c r="C212">
-        <v>97500000</v>
+        <v>113750000</v>
       </c>
       <c r="D212">
-        <v>6800000</v>
+        <v>3400000</v>
       </c>
       <c r="E212">
-        <v>71071407</v>
+        <v>74218210</v>
       </c>
       <c r="F212">
-        <v>77871407</v>
+        <v>77618210</v>
       </c>
       <c r="G212">
-        <v>19628593</v>
-      </c>
-      <c r="H212">
-        <v>32500000</v>
+        <v>36131790</v>
+      </c>
+      <c r="H212" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="213" spans="1:8" x14ac:dyDescent="0.3">
@@ -6845,16 +6852,16 @@
         <v>337500000</v>
       </c>
       <c r="D215">
-        <v>110694039</v>
+        <v>92956149</v>
       </c>
       <c r="E215">
-        <v>118245454</v>
+        <v>132840958</v>
       </c>
       <c r="F215">
-        <v>228939493</v>
+        <v>225797107</v>
       </c>
       <c r="G215">
-        <v>108560507</v>
+        <v>111702893</v>
       </c>
       <c r="H215">
         <v>112500000</v>
@@ -6871,10 +6878,10 @@
         <v>123750000</v>
       </c>
       <c r="D216">
-        <v>10000000</v>
+        <v>0</v>
       </c>
       <c r="E216">
-        <v>10900000</v>
+        <v>20900000</v>
       </c>
       <c r="F216">
         <v>20900000</v>
@@ -6891,25 +6898,25 @@
         <v>32</v>
       </c>
       <c r="B217">
-        <v>252000000</v>
+        <v>220500000</v>
       </c>
       <c r="C217">
-        <v>189000000</v>
+        <v>220500000</v>
       </c>
       <c r="D217">
         <v>0</v>
       </c>
       <c r="E217">
-        <v>169013000</v>
+        <v>170638000</v>
       </c>
       <c r="F217">
-        <v>169013000</v>
+        <v>170638000</v>
       </c>
       <c r="G217">
-        <v>19987000</v>
-      </c>
-      <c r="H217">
-        <v>63000000</v>
+        <v>49862000</v>
+      </c>
+      <c r="H217" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="218" spans="1:8" x14ac:dyDescent="0.3">
@@ -6978,13 +6985,13 @@
         <v>0</v>
       </c>
       <c r="E220">
-        <v>7090319905</v>
+        <v>7090340530</v>
       </c>
       <c r="F220">
-        <v>7090319905</v>
+        <v>7090340530</v>
       </c>
       <c r="G220">
-        <v>2732842221</v>
+        <v>2732821596</v>
       </c>
       <c r="H220" t="s">
         <v>9</v>
@@ -7027,10 +7034,10 @@
         <v>9245675372</v>
       </c>
       <c r="D222">
-        <v>29020768</v>
+        <v>0</v>
       </c>
       <c r="E222">
-        <v>8241279986</v>
+        <v>8270300754</v>
       </c>
       <c r="F222">
         <v>8270300754</v>
@@ -7131,10 +7138,10 @@
         <v>825165933</v>
       </c>
       <c r="D226">
-        <v>504035</v>
+        <v>0</v>
       </c>
       <c r="E226">
-        <v>1029675511</v>
+        <v>1030179546</v>
       </c>
       <c r="F226">
         <v>1030179546</v>
@@ -7177,25 +7184,25 @@
         <v>85</v>
       </c>
       <c r="B228">
-        <v>47914495045</v>
+        <v>47866745045</v>
       </c>
       <c r="C228">
-        <v>47499233545</v>
+        <v>47546983545</v>
       </c>
       <c r="D228">
-        <v>11457923938</v>
+        <v>11236071245</v>
       </c>
       <c r="E228">
-        <v>28822809671</v>
+        <v>28927242406</v>
       </c>
       <c r="F228">
-        <v>40280733609</v>
+        <v>40163313651</v>
       </c>
       <c r="G228">
-        <v>7218499936</v>
+        <v>7383669894</v>
       </c>
       <c r="H228">
-        <v>415261500</v>
+        <v>319761500</v>
       </c>
     </row>
     <row r="229" spans="1:8" x14ac:dyDescent="0.3">
@@ -7209,16 +7216,16 @@
         <v>12264606000</v>
       </c>
       <c r="D229">
-        <v>8206842730</v>
+        <v>8042712730</v>
       </c>
       <c r="E229">
-        <v>3238064000</v>
+        <v>3888767000</v>
       </c>
       <c r="F229">
-        <v>11444906730</v>
+        <v>11931479730</v>
       </c>
       <c r="G229">
-        <v>819699270</v>
+        <v>333126270</v>
       </c>
       <c r="H229" t="s">
         <v>9</v>
@@ -7235,10 +7242,10 @@
         <v>1126306000</v>
       </c>
       <c r="D230">
-        <v>1108174121</v>
+        <v>499624121</v>
       </c>
       <c r="E230">
-        <v>12436007</v>
+        <v>620986007</v>
       </c>
       <c r="F230">
         <v>1120610128</v>
@@ -7365,16 +7372,16 @@
         <v>1380000000</v>
       </c>
       <c r="D235">
-        <v>195458460</v>
+        <v>188118460</v>
       </c>
       <c r="E235">
         <v>1036121967</v>
       </c>
       <c r="F235">
-        <v>1231580427</v>
+        <v>1224240427</v>
       </c>
       <c r="G235">
-        <v>148419573</v>
+        <v>155759573</v>
       </c>
       <c r="H235" t="s">
         <v>9</v>
@@ -7732,13 +7739,13 @@
         <v>0</v>
       </c>
       <c r="E249">
-        <v>156115250</v>
+        <v>157565250</v>
       </c>
       <c r="F249">
-        <v>156115250</v>
+        <v>157565250</v>
       </c>
       <c r="G249">
-        <v>46168750</v>
+        <v>44718750</v>
       </c>
       <c r="H249">
         <v>67428000</v>
@@ -7784,13 +7791,13 @@
         <v>0</v>
       </c>
       <c r="E251">
-        <v>6996299227</v>
+        <v>6996336726</v>
       </c>
       <c r="F251">
-        <v>6996299227</v>
+        <v>6996336726</v>
       </c>
       <c r="G251">
-        <v>2829656943</v>
+        <v>2829619444</v>
       </c>
       <c r="H251" t="s">
         <v>9</v>
@@ -7833,10 +7840,10 @@
         <v>9512105917</v>
       </c>
       <c r="D253">
-        <v>27847073</v>
+        <v>0</v>
       </c>
       <c r="E253">
-        <v>8018348145</v>
+        <v>8046195218</v>
       </c>
       <c r="F253">
         <v>8046195218</v>
@@ -8015,16 +8022,16 @@
         <v>48914772555</v>
       </c>
       <c r="D260">
-        <v>11870059251</v>
+        <v>11062192178</v>
       </c>
       <c r="E260">
-        <v>28842124492</v>
+        <v>30130712064</v>
       </c>
       <c r="F260">
-        <v>40712183743</v>
+        <v>41192904242</v>
       </c>
       <c r="G260">
-        <v>8202588812</v>
+        <v>7721868313</v>
       </c>
       <c r="H260">
         <v>525212165</v>
@@ -8041,10 +8048,10 @@
         <v>5695069150</v>
       </c>
       <c r="D261">
-        <v>4255699600</v>
+        <v>3485289600</v>
       </c>
       <c r="E261">
-        <v>1346122000</v>
+        <v>2116532000</v>
       </c>
       <c r="F261">
         <v>5601821600</v>
@@ -8067,16 +8074,16 @@
         <v>1540000000</v>
       </c>
       <c r="D262">
-        <v>433950000</v>
+        <v>743352000</v>
       </c>
       <c r="E262">
         <v>784443706</v>
       </c>
       <c r="F262">
-        <v>1218393706</v>
+        <v>1527795706</v>
       </c>
       <c r="G262">
-        <v>321606294</v>
+        <v>12204294</v>
       </c>
       <c r="H262" t="s">
         <v>9</v>
@@ -8119,16 +8126,16 @@
         <v>150000000</v>
       </c>
       <c r="D264">
-        <v>0</v>
+        <v>137837144</v>
       </c>
       <c r="E264">
         <v>0</v>
       </c>
-      <c r="F264" t="s">
-        <v>9</v>
+      <c r="F264">
+        <v>137837144</v>
       </c>
       <c r="G264">
-        <v>150000000</v>
+        <v>12162856</v>
       </c>
       <c r="H264" t="s">
         <v>9</v>
@@ -8197,16 +8204,16 @@
         <v>491133000</v>
       </c>
       <c r="D267">
-        <v>0</v>
+        <v>388850000</v>
       </c>
       <c r="E267">
         <v>98325000</v>
       </c>
       <c r="F267">
-        <v>98325000</v>
+        <v>487175000</v>
       </c>
       <c r="G267">
-        <v>392808000</v>
+        <v>3958000</v>
       </c>
       <c r="H267" t="s">
         <v>9</v>
@@ -8223,16 +8230,16 @@
         <v>3609800000</v>
       </c>
       <c r="D268">
-        <v>1153620420</v>
+        <v>1660603451</v>
       </c>
       <c r="E268">
         <v>764581755</v>
       </c>
       <c r="F268">
-        <v>1918202175</v>
+        <v>2425185206</v>
       </c>
       <c r="G268">
-        <v>1691597825</v>
+        <v>1184614794</v>
       </c>
       <c r="H268" t="s">
         <v>9</v>
@@ -8535,16 +8542,16 @@
         <v>1242000000</v>
       </c>
       <c r="D280">
-        <v>922639865</v>
+        <v>878639865</v>
       </c>
       <c r="E280">
-        <v>47046943</v>
+        <v>90954943</v>
       </c>
       <c r="F280">
-        <v>969686808</v>
+        <v>969594808</v>
       </c>
       <c r="G280">
-        <v>272313192</v>
+        <v>272405192</v>
       </c>
       <c r="H280" t="s">
         <v>9</v>
@@ -8561,16 +8568,16 @@
         <v>150000000</v>
       </c>
       <c r="D281">
-        <v>121000000</v>
+        <v>0</v>
       </c>
       <c r="E281">
-        <v>0</v>
+        <v>120747000</v>
       </c>
       <c r="F281">
-        <v>121000000</v>
+        <v>120747000</v>
       </c>
       <c r="G281">
-        <v>29000000</v>
+        <v>29253000</v>
       </c>
       <c r="H281">
         <v>50000000</v>
@@ -8639,16 +8646,16 @@
         <v>235553350</v>
       </c>
       <c r="D284">
-        <v>7500000</v>
+        <v>107400000</v>
       </c>
       <c r="E284">
         <v>56925714</v>
       </c>
       <c r="F284">
-        <v>64425714</v>
+        <v>164325714</v>
       </c>
       <c r="G284">
-        <v>171127636</v>
+        <v>71227636</v>
       </c>
       <c r="H284">
         <v>20684450</v>
@@ -8665,16 +8672,16 @@
         <v>470406638</v>
       </c>
       <c r="D285">
-        <v>87270322</v>
+        <v>131370322</v>
       </c>
       <c r="E285">
         <v>282876433</v>
       </c>
       <c r="F285">
-        <v>370146755</v>
+        <v>414246755</v>
       </c>
       <c r="G285">
-        <v>100259883</v>
+        <v>56159883</v>
       </c>
       <c r="H285">
         <v>156802213</v>
@@ -8746,13 +8753,13 @@
         <v>0</v>
       </c>
       <c r="E288">
-        <v>212360250</v>
+        <v>212835250</v>
       </c>
       <c r="F288">
-        <v>212360250</v>
+        <v>212835250</v>
       </c>
       <c r="G288">
-        <v>136114000</v>
+        <v>135639000</v>
       </c>
       <c r="H288">
         <v>67824750</v>
@@ -8850,13 +8857,13 @@
         <v>0</v>
       </c>
       <c r="E292">
-        <v>8983834098</v>
+        <v>8983839723</v>
       </c>
       <c r="F292">
-        <v>8983834098</v>
+        <v>8983839723</v>
       </c>
       <c r="G292">
-        <v>3638784829</v>
+        <v>3638779204</v>
       </c>
       <c r="H292" t="s">
         <v>9</v>
@@ -8902,13 +8909,13 @@
         <v>0</v>
       </c>
       <c r="E294">
-        <v>10802659505</v>
+        <v>10841494695</v>
       </c>
       <c r="F294">
-        <v>10802659505</v>
+        <v>10841494695</v>
       </c>
       <c r="G294">
-        <v>2109057910</v>
+        <v>2070222720</v>
       </c>
       <c r="H294" t="s">
         <v>9</v>
@@ -9006,13 +9013,13 @@
         <v>0</v>
       </c>
       <c r="E298">
-        <v>1283180553</v>
+        <v>1283585105</v>
       </c>
       <c r="F298">
-        <v>1283180553</v>
+        <v>1283585105</v>
       </c>
       <c r="G298">
-        <v>277148284</v>
+        <v>276743732</v>
       </c>
       <c r="H298" t="s">
         <v>9</v>
@@ -9055,16 +9062,16 @@
         <v>63706784713</v>
       </c>
       <c r="D300">
-        <v>13985403855</v>
+        <v>14537066030</v>
       </c>
       <c r="E300">
-        <v>36266772843</v>
+        <v>37241558210</v>
       </c>
       <c r="F300">
-        <v>50252176698</v>
+        <v>51778624240</v>
       </c>
       <c r="G300">
-        <v>13454608015</v>
+        <v>11928160473</v>
       </c>
       <c r="H300">
         <v>531045413</v>
@@ -9081,10 +9088,10 @@
         <v>3628073000</v>
       </c>
       <c r="D301">
-        <v>1305682100</v>
+        <v>348213000</v>
       </c>
       <c r="E301">
-        <v>2322388900</v>
+        <v>3279858000</v>
       </c>
       <c r="F301">
         <v>3628071000</v>
@@ -9185,16 +9192,16 @@
         <v>298750000</v>
       </c>
       <c r="D305">
-        <v>228565327</v>
+        <v>232513230</v>
       </c>
       <c r="E305">
         <v>65826870</v>
       </c>
       <c r="F305">
-        <v>294392197</v>
+        <v>298340100</v>
       </c>
       <c r="G305">
-        <v>4357803</v>
+        <v>409900</v>
       </c>
       <c r="H305" t="s">
         <v>9</v>
@@ -9237,16 +9244,16 @@
         <v>1222108000</v>
       </c>
       <c r="D307">
-        <v>154177064</v>
+        <v>155107114</v>
       </c>
       <c r="E307">
         <v>1066657271</v>
       </c>
       <c r="F307">
-        <v>1220834335</v>
+        <v>1221764385</v>
       </c>
       <c r="G307">
-        <v>1273665</v>
+        <v>343615</v>
       </c>
       <c r="H307" t="s">
         <v>9</v>
@@ -9263,16 +9270,16 @@
         <v>534300000</v>
       </c>
       <c r="D308">
-        <v>130976265</v>
+        <v>140921415</v>
       </c>
       <c r="E308">
         <v>298405428</v>
       </c>
       <c r="F308">
-        <v>429381693</v>
+        <v>439326843</v>
       </c>
       <c r="G308">
-        <v>104918307</v>
+        <v>94973157</v>
       </c>
       <c r="H308" t="s">
         <v>9</v>
@@ -9315,16 +9322,16 @@
         <v>174000000</v>
       </c>
       <c r="D310">
-        <v>129869969</v>
+        <v>126215000</v>
       </c>
       <c r="E310">
         <v>44129340</v>
       </c>
       <c r="F310">
-        <v>173999309</v>
+        <v>170344340</v>
       </c>
       <c r="G310">
-        <v>691</v>
+        <v>3655660</v>
       </c>
       <c r="H310" t="s">
         <v>9</v>
@@ -9367,10 +9374,10 @@
         <v>1882400000</v>
       </c>
       <c r="D312">
-        <v>169090000</v>
+        <v>159330000</v>
       </c>
       <c r="E312">
-        <v>1713305000</v>
+        <v>1723065000</v>
       </c>
       <c r="F312">
         <v>1882395000</v>
@@ -9445,10 +9452,10 @@
         <v>463000000</v>
       </c>
       <c r="D315">
-        <v>388736000</v>
+        <v>353636000</v>
       </c>
       <c r="E315">
-        <v>45600000</v>
+        <v>80700000</v>
       </c>
       <c r="F315">
         <v>434336000</v>
@@ -9549,16 +9556,16 @@
         <v>64614000</v>
       </c>
       <c r="D319">
-        <v>20700400</v>
+        <v>22603358</v>
       </c>
       <c r="E319">
-        <v>24737271</v>
+        <v>26763571</v>
       </c>
       <c r="F319">
-        <v>45437671</v>
+        <v>49366929</v>
       </c>
       <c r="G319">
-        <v>19176329</v>
+        <v>15247071</v>
       </c>
       <c r="H319">
         <v>21538000</v>
@@ -9575,16 +9582,16 @@
         <v>82504500</v>
       </c>
       <c r="D320">
-        <v>8291500</v>
+        <v>12818500</v>
       </c>
       <c r="E320">
         <v>58799000</v>
       </c>
       <c r="F320">
-        <v>67090500</v>
+        <v>71617500</v>
       </c>
       <c r="G320">
-        <v>15414000</v>
+        <v>10887000</v>
       </c>
       <c r="H320">
         <v>27501500</v>
@@ -9757,10 +9764,10 @@
         <v>7015042421</v>
       </c>
       <c r="D327">
-        <v>19053817</v>
+        <v>0</v>
       </c>
       <c r="E327">
-        <v>5976157047</v>
+        <v>5995210864</v>
       </c>
       <c r="F327">
         <v>5995210864</v>
@@ -9861,10 +9868,10 @@
         <v>1449712379</v>
       </c>
       <c r="D331">
-        <v>608911</v>
+        <v>0</v>
       </c>
       <c r="E331">
-        <v>1144195047</v>
+        <v>1144803958</v>
       </c>
       <c r="F331">
         <v>1144803958</v>
@@ -9913,16 +9920,16 @@
         <v>30454436960</v>
       </c>
       <c r="D333">
-        <v>3303811758</v>
+        <v>2299418022</v>
       </c>
       <c r="E333">
-        <v>21478661365</v>
+        <v>22502679493</v>
       </c>
       <c r="F333">
-        <v>24782473123</v>
+        <v>24802097515</v>
       </c>
       <c r="G333">
-        <v>5671963837</v>
+        <v>5652339445</v>
       </c>
       <c r="H333">
         <v>260139500</v>
@@ -10017,10 +10024,10 @@
         <v>2593734264</v>
       </c>
       <c r="D337">
-        <v>1120961396</v>
+        <v>723018000</v>
       </c>
       <c r="E337">
-        <v>1472772814</v>
+        <v>1870716210</v>
       </c>
       <c r="F337">
         <v>2593734210</v>
@@ -10121,10 +10128,10 @@
         <v>1748195004</v>
       </c>
       <c r="D341">
-        <v>410290553</v>
+        <v>250654563</v>
       </c>
       <c r="E341">
-        <v>1202550785</v>
+        <v>1362186775</v>
       </c>
       <c r="F341">
         <v>1612841338</v>
@@ -10277,10 +10284,10 @@
         <v>150000000</v>
       </c>
       <c r="D347">
-        <v>143281590</v>
+        <v>100602000</v>
       </c>
       <c r="E347">
-        <v>0</v>
+        <v>42679590</v>
       </c>
       <c r="F347">
         <v>143281590</v>
@@ -10381,16 +10388,16 @@
         <v>571079775</v>
       </c>
       <c r="D351">
-        <v>241943670</v>
+        <v>262833670</v>
       </c>
       <c r="E351">
         <v>274818994</v>
       </c>
       <c r="F351">
-        <v>516762664</v>
+        <v>537652664</v>
       </c>
       <c r="G351">
-        <v>54317111</v>
+        <v>33427111</v>
       </c>
       <c r="H351">
         <v>190359925</v>
@@ -10433,16 +10440,16 @@
         <v>462375000</v>
       </c>
       <c r="D353">
-        <v>7253912</v>
+        <v>21419612</v>
       </c>
       <c r="E353">
         <v>331134371</v>
       </c>
       <c r="F353">
-        <v>338388283</v>
+        <v>352553983</v>
       </c>
       <c r="G353">
-        <v>123986717</v>
+        <v>109821017</v>
       </c>
       <c r="H353">
         <v>154125000</v>
@@ -10462,13 +10469,13 @@
         <v>0</v>
       </c>
       <c r="E354">
-        <v>167211500</v>
+        <v>169130250</v>
       </c>
       <c r="F354">
-        <v>167211500</v>
+        <v>169130250</v>
       </c>
       <c r="G354">
-        <v>93338500</v>
+        <v>91419750</v>
       </c>
       <c r="H354">
         <v>86850000</v>
@@ -10485,16 +10492,16 @@
         <v>6000000</v>
       </c>
       <c r="D355">
-        <v>467190</v>
+        <v>838020</v>
       </c>
       <c r="E355">
         <v>1500170</v>
       </c>
       <c r="F355">
-        <v>1967360</v>
+        <v>2338190</v>
       </c>
       <c r="G355">
-        <v>4032640</v>
+        <v>3661810</v>
       </c>
       <c r="H355" t="s">
         <v>9</v>
@@ -10540,13 +10547,13 @@
         <v>0</v>
       </c>
       <c r="E357">
-        <v>7461283668</v>
+        <v>7461330543</v>
       </c>
       <c r="F357">
-        <v>7461283668</v>
+        <v>7461330543</v>
       </c>
       <c r="G357">
-        <v>3253632345</v>
+        <v>3253585470</v>
       </c>
       <c r="H357" t="s">
         <v>9</v>
@@ -10589,16 +10596,16 @@
         <v>10532164202</v>
       </c>
       <c r="D359">
-        <v>0</v>
+        <v>32608180</v>
       </c>
       <c r="E359">
         <v>8834277017</v>
       </c>
       <c r="F359">
-        <v>8834277017</v>
+        <v>8866885197</v>
       </c>
       <c r="G359">
-        <v>1697887185</v>
+        <v>1665279005</v>
       </c>
       <c r="H359" t="s">
         <v>9</v>
@@ -10693,16 +10700,16 @@
         <v>1523018104</v>
       </c>
       <c r="D363">
-        <v>0</v>
+        <v>811692</v>
       </c>
       <c r="E363">
         <v>1236176601</v>
       </c>
       <c r="F363">
-        <v>1236176601</v>
+        <v>1236988293</v>
       </c>
       <c r="G363">
-        <v>286841503</v>
+        <v>286029811</v>
       </c>
       <c r="H363" t="s">
         <v>9</v>
@@ -10745,16 +10752,16 @@
         <v>57427089299</v>
       </c>
       <c r="D365">
-        <v>8890841939</v>
+        <v>8359429365</v>
       </c>
       <c r="E365">
-        <v>40908452881</v>
+        <v>41510677482</v>
       </c>
       <c r="F365">
-        <v>49799294820</v>
+        <v>49870106847</v>
       </c>
       <c r="G365">
-        <v>7627794479</v>
+        <v>7556982452</v>
       </c>
       <c r="H365">
         <v>526334925</v>
@@ -10849,16 +10856,16 @@
         <v>2467762918</v>
       </c>
       <c r="D369">
-        <v>1217556059</v>
+        <v>1755568584</v>
       </c>
       <c r="E369">
         <v>558800786</v>
       </c>
       <c r="F369">
-        <v>1776356845</v>
+        <v>2314369370</v>
       </c>
       <c r="G369">
-        <v>691406073</v>
+        <v>153393548</v>
       </c>
       <c r="H369" t="s">
         <v>9</v>
@@ -10927,16 +10934,16 @@
         <v>1714789867</v>
       </c>
       <c r="D372">
-        <v>920522269</v>
+        <v>951703341</v>
       </c>
       <c r="E372">
         <v>732962308</v>
       </c>
       <c r="F372">
-        <v>1653484577</v>
+        <v>1684665649</v>
       </c>
       <c r="G372">
-        <v>61305290</v>
+        <v>30124218</v>
       </c>
       <c r="H372" t="s">
         <v>9</v>
@@ -10979,16 +10986,16 @@
         <v>290550000</v>
       </c>
       <c r="D374">
-        <v>290377764</v>
+        <v>290264873</v>
       </c>
       <c r="E374">
         <v>0</v>
       </c>
       <c r="F374">
-        <v>290377764</v>
+        <v>290264873</v>
       </c>
       <c r="G374">
-        <v>172236</v>
+        <v>285127</v>
       </c>
       <c r="H374" t="s">
         <v>9</v>
@@ -11031,16 +11038,16 @@
         <v>470200000</v>
       </c>
       <c r="D376">
-        <v>45290400</v>
+        <v>0</v>
       </c>
       <c r="E376">
         <v>424909600</v>
       </c>
       <c r="F376">
-        <v>470200000</v>
-      </c>
-      <c r="G376" t="s">
-        <v>9</v>
+        <v>424909600</v>
+      </c>
+      <c r="G376">
+        <v>45290400</v>
       </c>
       <c r="H376" t="s">
         <v>9</v>
@@ -11057,16 +11064,16 @@
         <v>200000000</v>
       </c>
       <c r="D377">
-        <v>150079500</v>
+        <v>147528500</v>
       </c>
       <c r="E377">
         <v>49920000</v>
       </c>
       <c r="F377">
-        <v>199999500</v>
+        <v>197448500</v>
       </c>
       <c r="G377">
-        <v>500</v>
+        <v>2551500</v>
       </c>
       <c r="H377" t="s">
         <v>9</v>
@@ -11083,16 +11090,16 @@
         <v>82500000</v>
       </c>
       <c r="D378">
-        <v>77719680</v>
+        <v>0</v>
       </c>
       <c r="E378">
-        <v>0</v>
+        <v>76086680</v>
       </c>
       <c r="F378">
-        <v>77719680</v>
+        <v>76086680</v>
       </c>
       <c r="G378">
-        <v>4780320</v>
+        <v>6413320</v>
       </c>
       <c r="H378">
         <v>27500000</v>
@@ -11135,10 +11142,10 @@
         <v>411080000</v>
       </c>
       <c r="D380">
-        <v>1827440</v>
+        <v>489790</v>
       </c>
       <c r="E380">
-        <v>279958254</v>
+        <v>281295904</v>
       </c>
       <c r="F380">
         <v>281785694</v>
@@ -11187,10 +11194,10 @@
         <v>300000000</v>
       </c>
       <c r="D382">
-        <v>79412000</v>
+        <v>67912000</v>
       </c>
       <c r="E382">
-        <v>183314712</v>
+        <v>194814712</v>
       </c>
       <c r="F382">
         <v>262726712</v>
@@ -11268,13 +11275,13 @@
         <v>0</v>
       </c>
       <c r="E385">
-        <v>110610500</v>
+        <v>124406000</v>
       </c>
       <c r="F385">
-        <v>110610500</v>
+        <v>124406000</v>
       </c>
       <c r="G385">
-        <v>17414500</v>
+        <v>3619000</v>
       </c>
       <c r="H385">
         <v>42675000</v>
@@ -11372,13 +11379,13 @@
         <v>0</v>
       </c>
       <c r="E389">
-        <v>3205079550</v>
+        <v>3205993500</v>
       </c>
       <c r="F389">
-        <v>3205079550</v>
+        <v>3205993500</v>
       </c>
       <c r="G389">
-        <v>1334727368</v>
+        <v>1333813418</v>
       </c>
       <c r="H389" t="s">
         <v>9</v>
@@ -11577,16 +11584,16 @@
         <v>24628424376</v>
       </c>
       <c r="D397">
-        <v>4529784150</v>
+        <v>4960466126</v>
       </c>
       <c r="E397">
-        <v>15449970210</v>
+        <v>15553603990</v>
       </c>
       <c r="F397">
-        <v>19979754360</v>
+        <v>20514070116</v>
       </c>
       <c r="G397">
-        <v>4648670016</v>
+        <v>4114354260</v>
       </c>
       <c r="H397">
         <v>232675000</v>
@@ -12019,16 +12026,16 @@
         <v>2230000000</v>
       </c>
       <c r="D414">
-        <v>19000000</v>
+        <v>9815000</v>
       </c>
       <c r="E414">
-        <v>1017375537</v>
+        <v>1025934097</v>
       </c>
       <c r="F414">
-        <v>1036375537</v>
+        <v>1035749097</v>
       </c>
       <c r="G414">
-        <v>1193624463</v>
+        <v>1194250903</v>
       </c>
       <c r="H414" t="s">
         <v>9</v>
@@ -12045,10 +12052,10 @@
         <v>145200000</v>
       </c>
       <c r="D415">
-        <v>30647800</v>
+        <v>22211800</v>
       </c>
       <c r="E415">
-        <v>67309500</v>
+        <v>75745500</v>
       </c>
       <c r="F415">
         <v>97957300</v>
@@ -12305,16 +12312,16 @@
         <v>9379568492</v>
       </c>
       <c r="D425">
-        <v>0</v>
+        <v>26591563</v>
       </c>
       <c r="E425">
         <v>7295042089</v>
       </c>
       <c r="F425">
-        <v>7295042089</v>
+        <v>7321633652</v>
       </c>
       <c r="G425">
-        <v>2084526403</v>
+        <v>2057934840</v>
       </c>
       <c r="H425" t="s">
         <v>9</v>
@@ -12461,16 +12468,16 @@
         <v>35458361640</v>
       </c>
       <c r="D431">
-        <v>5477255293</v>
+        <v>5486225856</v>
       </c>
       <c r="E431">
-        <v>21346375474</v>
+        <v>21363370034</v>
       </c>
       <c r="F431">
-        <v>26823630767</v>
+        <v>26849595890</v>
       </c>
       <c r="G431">
-        <v>8634730873</v>
+        <v>8608765750</v>
       </c>
       <c r="H431">
         <v>472807750</v>
@@ -12480,128 +12487,241 @@
       <c r="A432" t="s">
         <v>8</v>
       </c>
-      <c r="B432">
+      <c r="B432" s="1">
         <v>873740000</v>
       </c>
-      <c r="C432">
+      <c r="C432" s="1">
         <v>873740000</v>
       </c>
-      <c r="D432">
+      <c r="D432" s="1">
         <v>255557500</v>
       </c>
-      <c r="E432">
+      <c r="E432" s="1">
         <v>589750552</v>
       </c>
-      <c r="F432">
+      <c r="F432" s="1">
         <v>845308052</v>
       </c>
-      <c r="G432">
+      <c r="G432" s="1">
         <v>28431948</v>
       </c>
-      <c r="H432">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="433" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="H432" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="433" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A433" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="434" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B433" s="1"/>
+      <c r="C433" s="1"/>
+      <c r="D433" s="1"/>
+      <c r="E433" s="1"/>
+      <c r="F433" s="1"/>
+      <c r="G433" s="1"/>
+      <c r="H433" s="1"/>
+    </row>
+    <row r="434" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A434" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="435" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B434" s="1"/>
+      <c r="C434" s="1"/>
+      <c r="D434" s="1"/>
+      <c r="E434" s="1"/>
+      <c r="F434" s="1"/>
+      <c r="G434" s="1"/>
+      <c r="H434" s="1"/>
+    </row>
+    <row r="435" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A435" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="436" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B435" s="1"/>
+      <c r="C435" s="1"/>
+      <c r="D435" s="1"/>
+      <c r="E435" s="1"/>
+      <c r="F435" s="1"/>
+      <c r="G435" s="1"/>
+      <c r="H435" s="1"/>
+    </row>
+    <row r="436" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A436" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="437" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B436" s="1"/>
+      <c r="C436" s="1"/>
+      <c r="D436" s="1"/>
+      <c r="E436" s="1"/>
+      <c r="F436" s="1"/>
+      <c r="G436" s="1"/>
+      <c r="H436" s="1"/>
+    </row>
+    <row r="437" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A437" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="438" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B437" s="1"/>
+      <c r="C437" s="1"/>
+      <c r="D437" s="1"/>
+      <c r="E437" s="1"/>
+      <c r="F437" s="1"/>
+      <c r="G437" s="1"/>
+      <c r="H437" s="1"/>
+    </row>
+    <row r="438" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A438" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="439" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B438" s="1"/>
+      <c r="C438" s="1"/>
+      <c r="D438" s="1"/>
+      <c r="E438" s="1"/>
+      <c r="F438" s="1"/>
+      <c r="G438" s="1"/>
+      <c r="H438" s="1"/>
+    </row>
+    <row r="439" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A439" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="440" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B439" s="1"/>
+      <c r="C439" s="1"/>
+      <c r="D439" s="1"/>
+      <c r="E439" s="1"/>
+      <c r="F439" s="1"/>
+      <c r="G439" s="1"/>
+      <c r="H439" s="1"/>
+    </row>
+    <row r="440" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A440" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="441" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B440" s="1"/>
+      <c r="C440" s="1"/>
+      <c r="D440" s="1"/>
+      <c r="E440" s="1"/>
+      <c r="F440" s="1"/>
+      <c r="G440" s="1"/>
+      <c r="H440" s="1"/>
+    </row>
+    <row r="441" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A441" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="442" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B441" s="1"/>
+      <c r="C441" s="1"/>
+      <c r="D441" s="1"/>
+      <c r="E441" s="1"/>
+      <c r="F441" s="1"/>
+      <c r="G441" s="1"/>
+      <c r="H441" s="1"/>
+    </row>
+    <row r="442" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A442" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="443" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B442" s="1"/>
+      <c r="C442" s="1"/>
+      <c r="D442" s="1"/>
+      <c r="E442" s="1"/>
+      <c r="F442" s="1"/>
+      <c r="G442" s="1"/>
+      <c r="H442" s="1"/>
+    </row>
+    <row r="443" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A443" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="444" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B443" s="1"/>
+      <c r="C443" s="1"/>
+      <c r="D443" s="1"/>
+      <c r="E443" s="1"/>
+      <c r="F443" s="1"/>
+      <c r="G443" s="1"/>
+      <c r="H443" s="1"/>
+    </row>
+    <row r="444" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A444" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="445" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B444" s="1"/>
+      <c r="C444" s="1"/>
+      <c r="D444" s="1"/>
+      <c r="E444" s="1"/>
+      <c r="F444" s="1"/>
+      <c r="G444" s="1"/>
+      <c r="H444" s="1"/>
+    </row>
+    <row r="445" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A445" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="446" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B445" s="1"/>
+      <c r="C445" s="1"/>
+      <c r="D445" s="1"/>
+      <c r="E445" s="1"/>
+      <c r="F445" s="1"/>
+      <c r="G445" s="1"/>
+      <c r="H445" s="1"/>
+    </row>
+    <row r="446" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A446" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="447" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B446" s="1"/>
+      <c r="C446" s="1"/>
+      <c r="D446" s="1"/>
+      <c r="E446" s="1"/>
+      <c r="F446" s="1"/>
+      <c r="G446" s="1"/>
+      <c r="H446" s="1"/>
+    </row>
+    <row r="447" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A447" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="448" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B447" s="1"/>
+      <c r="C447" s="1"/>
+      <c r="D447" s="1"/>
+      <c r="E447" s="1"/>
+      <c r="F447" s="1"/>
+      <c r="G447" s="1"/>
+      <c r="H447" s="1"/>
+    </row>
+    <row r="448" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A448" t="s">
         <v>107</v>
       </c>
+      <c r="B448" s="1"/>
+      <c r="C448" s="1"/>
+      <c r="D448" s="1"/>
+      <c r="E448" s="1"/>
+      <c r="F448" s="1"/>
+      <c r="G448" s="1"/>
+      <c r="H448" s="1"/>
     </row>
     <row r="449" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A449" t="s">
         <v>55</v>
       </c>
-      <c r="B449">
+      <c r="B449" s="1">
         <v>474786000</v>
       </c>
-      <c r="C449">
+      <c r="C449" s="1">
         <v>474786000</v>
       </c>
-      <c r="D449">
+      <c r="D449" s="1">
         <v>474154600</v>
       </c>
-      <c r="F449">
+      <c r="E449" s="1"/>
+      <c r="F449" s="1">
         <v>474154600</v>
       </c>
-      <c r="G449">
+      <c r="G449" s="1">
         <v>631400</v>
       </c>
-      <c r="H449">
+      <c r="H449" s="1">
         <v>0</v>
       </c>
     </row>
@@ -12609,22 +12729,23 @@
       <c r="A450" t="s">
         <v>14</v>
       </c>
-      <c r="B450">
+      <c r="B450" s="1">
         <v>208424730</v>
       </c>
-      <c r="C450">
+      <c r="C450" s="1">
         <v>208424730</v>
       </c>
-      <c r="D450">
+      <c r="D450" s="1">
         <v>180590600</v>
       </c>
-      <c r="F450">
+      <c r="E450" s="1"/>
+      <c r="F450" s="1">
         <v>180590600</v>
       </c>
-      <c r="G450">
+      <c r="G450" s="1">
         <v>27834130</v>
       </c>
-      <c r="H450">
+      <c r="H450" s="1">
         <v>0</v>
       </c>
     </row>
@@ -12632,25 +12753,25 @@
       <c r="A451" t="s">
         <v>16</v>
       </c>
-      <c r="B451">
+      <c r="B451" s="1">
         <v>20000000</v>
       </c>
-      <c r="C451">
+      <c r="C451" s="1">
         <v>20000000</v>
       </c>
-      <c r="D451">
-        <v>0</v>
-      </c>
-      <c r="E451">
+      <c r="D451" s="1">
+        <v>0</v>
+      </c>
+      <c r="E451" s="1">
         <v>13970000</v>
       </c>
-      <c r="F451">
+      <c r="F451" s="1">
         <v>13970000</v>
       </c>
-      <c r="G451">
+      <c r="G451" s="1">
         <v>6030000</v>
       </c>
-      <c r="H451">
+      <c r="H451" s="1">
         <v>0</v>
       </c>
     </row>
@@ -12658,25 +12779,25 @@
       <c r="A452" t="s">
         <v>17</v>
       </c>
-      <c r="B452">
+      <c r="B452" s="1">
         <v>220000000</v>
       </c>
-      <c r="C452">
+      <c r="C452" s="1">
         <v>220000000</v>
       </c>
-      <c r="D452">
+      <c r="D452" s="1">
         <v>48700000</v>
       </c>
-      <c r="E452">
+      <c r="E452" s="1">
         <v>89688678</v>
       </c>
-      <c r="F452">
+      <c r="F452" s="1">
         <v>138388678</v>
       </c>
-      <c r="G452">
+      <c r="G452" s="1">
         <v>81611322</v>
       </c>
-      <c r="H452">
+      <c r="H452" s="1">
         <v>0</v>
       </c>
     </row>
@@ -12684,22 +12805,23 @@
       <c r="A453" t="s">
         <v>59</v>
       </c>
-      <c r="B453">
+      <c r="B453" s="1">
         <v>75000000</v>
       </c>
-      <c r="C453">
+      <c r="C453" s="1">
         <v>75000000</v>
       </c>
-      <c r="D453">
+      <c r="D453" s="1">
         <v>38500000</v>
       </c>
-      <c r="F453">
+      <c r="E453" s="1"/>
+      <c r="F453" s="1">
         <v>38500000</v>
       </c>
-      <c r="G453">
+      <c r="G453" s="1">
         <v>36500000</v>
       </c>
-      <c r="H453">
+      <c r="H453" s="1">
         <v>0</v>
       </c>
     </row>
@@ -12707,35 +12829,49 @@
       <c r="A454" t="s">
         <v>108</v>
       </c>
+      <c r="B454" s="1"/>
+      <c r="C454" s="1"/>
+      <c r="D454" s="1"/>
+      <c r="E454" s="1"/>
+      <c r="F454" s="1"/>
+      <c r="G454" s="1"/>
+      <c r="H454" s="1"/>
     </row>
     <row r="455" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A455" t="s">
         <v>109</v>
       </c>
+      <c r="B455" s="1"/>
+      <c r="C455" s="1"/>
+      <c r="D455" s="1"/>
+      <c r="E455" s="1"/>
+      <c r="F455" s="1"/>
+      <c r="G455" s="1"/>
+      <c r="H455" s="1"/>
     </row>
     <row r="456" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A456" t="s">
         <v>24</v>
       </c>
-      <c r="B456">
+      <c r="B456" s="1">
         <v>60000000</v>
       </c>
-      <c r="C456">
+      <c r="C456" s="1">
         <v>45000000</v>
       </c>
-      <c r="D456">
+      <c r="D456" s="1">
         <v>7388000</v>
       </c>
-      <c r="E456">
+      <c r="E456" s="1">
         <v>10120000</v>
       </c>
-      <c r="F456">
+      <c r="F456" s="1">
         <v>17508000</v>
       </c>
-      <c r="G456">
+      <c r="G456" s="1">
         <v>27492000</v>
       </c>
-      <c r="H456">
+      <c r="H456" s="1">
         <v>15000000</v>
       </c>
     </row>
@@ -12743,25 +12879,25 @@
       <c r="A457" t="s">
         <v>64</v>
       </c>
-      <c r="B457">
+      <c r="B457" s="1">
         <v>45150000</v>
       </c>
-      <c r="C457">
+      <c r="C457" s="1">
         <v>45150000</v>
       </c>
-      <c r="D457">
+      <c r="D457" s="1">
         <v>7130850</v>
       </c>
-      <c r="E457">
+      <c r="E457" s="1">
         <v>20796200</v>
       </c>
-      <c r="F457">
+      <c r="F457" s="1">
         <v>27927050</v>
       </c>
-      <c r="G457">
+      <c r="G457" s="1">
         <v>17222950</v>
       </c>
-      <c r="H457">
+      <c r="H457" s="1">
         <v>0</v>
       </c>
     </row>
@@ -12769,64 +12905,129 @@
       <c r="A458" t="s">
         <v>25</v>
       </c>
+      <c r="B458" s="1"/>
+      <c r="C458" s="1"/>
+      <c r="D458" s="1"/>
+      <c r="E458" s="1"/>
+      <c r="F458" s="1"/>
+      <c r="G458" s="1"/>
+      <c r="H458" s="1"/>
     </row>
     <row r="459" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A459" t="s">
         <v>110</v>
       </c>
+      <c r="B459" s="1"/>
+      <c r="C459" s="1"/>
+      <c r="D459" s="1"/>
+      <c r="E459" s="1"/>
+      <c r="F459" s="1"/>
+      <c r="G459" s="1"/>
+      <c r="H459" s="1"/>
     </row>
     <row r="460" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A460" t="s">
         <v>111</v>
       </c>
+      <c r="B460" s="1"/>
+      <c r="C460" s="1"/>
+      <c r="D460" s="1"/>
+      <c r="E460" s="1"/>
+      <c r="F460" s="1"/>
+      <c r="G460" s="1"/>
+      <c r="H460" s="1"/>
     </row>
     <row r="461" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A461" t="s">
         <v>112</v>
       </c>
+      <c r="B461" s="1"/>
+      <c r="C461" s="1"/>
+      <c r="D461" s="1"/>
+      <c r="E461" s="1"/>
+      <c r="F461" s="1"/>
+      <c r="G461" s="1"/>
+      <c r="H461" s="1"/>
     </row>
     <row r="462" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A462" t="s">
         <v>113</v>
       </c>
+      <c r="B462" s="1"/>
+      <c r="C462" s="1"/>
+      <c r="D462" s="1"/>
+      <c r="E462" s="1"/>
+      <c r="F462" s="1"/>
+      <c r="G462" s="1"/>
+      <c r="H462" s="1"/>
     </row>
     <row r="463" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A463" t="s">
         <v>114</v>
       </c>
+      <c r="B463" s="1"/>
+      <c r="C463" s="1"/>
+      <c r="D463" s="1"/>
+      <c r="E463" s="1"/>
+      <c r="F463" s="1"/>
+      <c r="G463" s="1"/>
+      <c r="H463" s="1"/>
     </row>
     <row r="464" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A464" t="s">
         <v>115</v>
       </c>
+      <c r="B464" s="1"/>
+      <c r="C464" s="1"/>
+      <c r="D464" s="1"/>
+      <c r="E464" s="1"/>
+      <c r="F464" s="1"/>
+      <c r="G464" s="1"/>
+      <c r="H464" s="1"/>
     </row>
     <row r="465" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A465" t="s">
         <v>116</v>
       </c>
+      <c r="B465" s="1"/>
+      <c r="C465" s="1"/>
+      <c r="D465" s="1"/>
+      <c r="E465" s="1"/>
+      <c r="F465" s="1"/>
+      <c r="G465" s="1"/>
+      <c r="H465" s="1"/>
     </row>
     <row r="466" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A466" t="s">
         <v>117</v>
       </c>
+      <c r="B466" s="1"/>
+      <c r="C466" s="1"/>
+      <c r="D466" s="1"/>
+      <c r="E466" s="1"/>
+      <c r="F466" s="1"/>
+      <c r="G466" s="1"/>
+      <c r="H466" s="1"/>
     </row>
     <row r="467" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A467" t="s">
         <v>27</v>
       </c>
-      <c r="B467">
+      <c r="B467" s="1">
         <v>6000000</v>
       </c>
-      <c r="C467">
+      <c r="C467" s="1">
         <v>4500000</v>
       </c>
-      <c r="D467">
-        <v>0</v>
-      </c>
-      <c r="G467">
+      <c r="D467" s="1">
+        <v>0</v>
+      </c>
+      <c r="E467" s="1"/>
+      <c r="F467" s="1"/>
+      <c r="G467" s="1">
         <v>4500000</v>
       </c>
-      <c r="H467">
+      <c r="H467" s="1">
         <v>1500000</v>
       </c>
     </row>
@@ -12834,25 +13035,25 @@
       <c r="A468" t="s">
         <v>28</v>
       </c>
-      <c r="B468">
+      <c r="B468" s="1">
         <v>41000000</v>
       </c>
-      <c r="C468">
+      <c r="C468" s="1">
         <v>30750000</v>
       </c>
-      <c r="D468">
+      <c r="D468" s="1">
         <v>6869550</v>
       </c>
-      <c r="E468">
+      <c r="E468" s="1">
         <v>4982700</v>
       </c>
-      <c r="F468">
+      <c r="F468" s="1">
         <v>11852250</v>
       </c>
-      <c r="G468">
+      <c r="G468" s="1">
         <v>18897750</v>
       </c>
-      <c r="H468">
+      <c r="H468" s="1">
         <v>10250000</v>
       </c>
     </row>
@@ -12860,19 +13061,21 @@
       <c r="A469" t="s">
         <v>29</v>
       </c>
-      <c r="B469">
+      <c r="B469" s="1">
         <v>12000000</v>
       </c>
-      <c r="C469">
+      <c r="C469" s="1">
         <v>3000000</v>
       </c>
-      <c r="D469">
-        <v>0</v>
-      </c>
-      <c r="G469">
+      <c r="D469" s="1">
+        <v>0</v>
+      </c>
+      <c r="E469" s="1"/>
+      <c r="F469" s="1"/>
+      <c r="G469" s="1">
         <v>3000000</v>
       </c>
-      <c r="H469">
+      <c r="H469" s="1">
         <v>9000000</v>
       </c>
     </row>
@@ -12880,25 +13083,25 @@
       <c r="A470" t="s">
         <v>30</v>
       </c>
-      <c r="B470">
+      <c r="B470" s="1">
         <v>171000000</v>
       </c>
-      <c r="C470">
+      <c r="C470" s="1">
         <v>128250000</v>
       </c>
-      <c r="D470">
+      <c r="D470" s="1">
         <v>17585000</v>
       </c>
-      <c r="E470">
+      <c r="E470" s="1">
         <v>20876000</v>
       </c>
-      <c r="F470">
+      <c r="F470" s="1">
         <v>38461000</v>
       </c>
-      <c r="G470">
+      <c r="G470" s="1">
         <v>89789000</v>
       </c>
-      <c r="H470">
+      <c r="H470" s="1">
         <v>42750000</v>
       </c>
     </row>
@@ -12906,25 +13109,25 @@
       <c r="A471" t="s">
         <v>32</v>
       </c>
-      <c r="B471">
+      <c r="B471" s="1">
         <v>130000000</v>
       </c>
-      <c r="C471">
+      <c r="C471" s="1">
         <v>97500000</v>
       </c>
-      <c r="D471">
+      <c r="D471" s="1">
         <v>23953308</v>
       </c>
-      <c r="E471">
+      <c r="E471" s="1">
         <v>59537750</v>
       </c>
-      <c r="F471">
+      <c r="F471" s="1">
         <v>83491058</v>
       </c>
-      <c r="G471">
+      <c r="G471" s="1">
         <v>14008942</v>
       </c>
-      <c r="H471">
+      <c r="H471" s="1">
         <v>32500000</v>
       </c>
     </row>
@@ -12932,25 +13135,25 @@
       <c r="A472" t="s">
         <v>84</v>
       </c>
-      <c r="B472">
+      <c r="B472" s="1">
         <v>6660000</v>
       </c>
-      <c r="C472">
+      <c r="C472" s="1">
         <v>6660000</v>
       </c>
-      <c r="D472">
+      <c r="D472" s="1">
         <v>2240000</v>
       </c>
-      <c r="E472">
+      <c r="E472" s="1">
         <v>4246644</v>
       </c>
-      <c r="F472">
+      <c r="F472" s="1">
         <v>6486644</v>
       </c>
-      <c r="G472">
+      <c r="G472" s="1">
         <v>173356</v>
       </c>
-      <c r="H472">
+      <c r="H472" s="1">
         <v>0</v>
       </c>
     </row>
@@ -12958,25 +13161,25 @@
       <c r="A473" t="s">
         <v>33</v>
       </c>
-      <c r="B473">
+      <c r="B473" s="1">
         <v>6000000</v>
       </c>
-      <c r="C473">
+      <c r="C473" s="1">
         <v>6000000</v>
       </c>
-      <c r="D473">
-        <v>0</v>
-      </c>
-      <c r="E473">
+      <c r="D473" s="1">
+        <v>0</v>
+      </c>
+      <c r="E473" s="1">
         <v>5982000</v>
       </c>
-      <c r="F473">
+      <c r="F473" s="1">
         <v>5982000</v>
       </c>
-      <c r="G473">
+      <c r="G473" s="1">
         <v>18000</v>
       </c>
-      <c r="H473">
+      <c r="H473" s="1">
         <v>0</v>
       </c>
     </row>
@@ -12984,71 +13187,169 @@
       <c r="A474" t="s">
         <v>78</v>
       </c>
+      <c r="B474" s="1"/>
+      <c r="C474" s="1"/>
+      <c r="D474" s="1"/>
+      <c r="E474" s="1"/>
+      <c r="F474" s="1"/>
+      <c r="G474" s="1"/>
+      <c r="H474" s="1"/>
     </row>
     <row r="475" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A475" t="s">
         <v>66</v>
       </c>
+      <c r="B475" s="1"/>
+      <c r="C475" s="1"/>
+      <c r="D475" s="1"/>
+      <c r="E475" s="1"/>
+      <c r="F475" s="1"/>
+      <c r="G475" s="1"/>
+      <c r="H475" s="1"/>
     </row>
     <row r="476" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A476" t="s">
         <v>34</v>
       </c>
+      <c r="B476" s="1"/>
+      <c r="C476" s="1"/>
+      <c r="D476" s="1"/>
+      <c r="E476" s="1"/>
+      <c r="F476" s="1"/>
+      <c r="G476" s="1"/>
+      <c r="H476" s="1"/>
     </row>
     <row r="477" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A477" t="s">
         <v>79</v>
       </c>
+      <c r="B477" s="1"/>
+      <c r="C477" s="1"/>
+      <c r="D477" s="1"/>
+      <c r="E477" s="1"/>
+      <c r="F477" s="1"/>
+      <c r="G477" s="1"/>
+      <c r="H477" s="1"/>
     </row>
     <row r="478" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A478" t="s">
         <v>118</v>
       </c>
+      <c r="B478" s="1"/>
+      <c r="C478" s="1"/>
+      <c r="D478" s="1"/>
+      <c r="E478" s="1"/>
+      <c r="F478" s="1"/>
+      <c r="G478" s="1"/>
+      <c r="H478" s="1"/>
     </row>
     <row r="479" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A479" t="s">
         <v>35</v>
       </c>
+      <c r="B479" s="1"/>
+      <c r="C479" s="1"/>
+      <c r="D479" s="1"/>
+      <c r="E479" s="1"/>
+      <c r="F479" s="1"/>
+      <c r="G479" s="1"/>
+      <c r="H479" s="1"/>
     </row>
     <row r="480" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A480" t="s">
         <v>36</v>
       </c>
+      <c r="B480" s="1"/>
+      <c r="C480" s="1"/>
+      <c r="D480" s="1"/>
+      <c r="E480" s="1"/>
+      <c r="F480" s="1"/>
+      <c r="G480" s="1"/>
+      <c r="H480" s="1"/>
     </row>
     <row r="481" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A481" t="s">
         <v>37</v>
       </c>
+      <c r="B481" s="1"/>
+      <c r="C481" s="1"/>
+      <c r="D481" s="1"/>
+      <c r="E481" s="1"/>
+      <c r="F481" s="1"/>
+      <c r="G481" s="1"/>
+      <c r="H481" s="1"/>
     </row>
     <row r="482" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A482" t="s">
         <v>38</v>
       </c>
+      <c r="B482" s="1"/>
+      <c r="C482" s="1"/>
+      <c r="D482" s="1"/>
+      <c r="E482" s="1"/>
+      <c r="F482" s="1"/>
+      <c r="G482" s="1"/>
+      <c r="H482" s="1"/>
     </row>
     <row r="483" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A483" t="s">
         <v>39</v>
       </c>
+      <c r="B483" s="1"/>
+      <c r="C483" s="1"/>
+      <c r="D483" s="1"/>
+      <c r="E483" s="1"/>
+      <c r="F483" s="1"/>
+      <c r="G483" s="1"/>
+      <c r="H483" s="1"/>
     </row>
     <row r="484" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A484" t="s">
         <v>41</v>
       </c>
+      <c r="B484" s="1"/>
+      <c r="C484" s="1"/>
+      <c r="D484" s="1"/>
+      <c r="E484" s="1"/>
+      <c r="F484" s="1"/>
+      <c r="G484" s="1"/>
+      <c r="H484" s="1"/>
     </row>
     <row r="485" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A485" t="s">
         <v>42</v>
       </c>
+      <c r="B485" s="1"/>
+      <c r="C485" s="1"/>
+      <c r="D485" s="1"/>
+      <c r="E485" s="1"/>
+      <c r="F485" s="1"/>
+      <c r="G485" s="1"/>
+      <c r="H485" s="1"/>
     </row>
     <row r="486" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A486" t="s">
         <v>48</v>
       </c>
+      <c r="B486" s="1"/>
+      <c r="C486" s="1"/>
+      <c r="D486" s="1"/>
+      <c r="E486" s="1"/>
+      <c r="F486" s="1"/>
+      <c r="G486" s="1"/>
+      <c r="H486" s="1"/>
     </row>
     <row r="487" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A487" t="s">
         <v>119</v>
       </c>
+      <c r="B487" s="1"/>
+      <c r="C487" s="1"/>
+      <c r="D487" s="1"/>
+      <c r="E487" s="1"/>
+      <c r="F487" s="1"/>
+      <c r="G487" s="1"/>
+      <c r="H487" s="1"/>
     </row>
     <row r="488" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A488" t="s">
@@ -13243,16 +13544,16 @@
         <v>2312795000</v>
       </c>
       <c r="D495">
-        <v>1294531850</v>
+        <v>1255550010</v>
       </c>
       <c r="E495">
-        <v>605293954</v>
+        <v>654993954</v>
       </c>
       <c r="F495">
-        <v>1899825804</v>
+        <v>1910543964</v>
       </c>
       <c r="G495">
-        <v>412969196</v>
+        <v>402251036</v>
       </c>
       <c r="H495" t="s">
         <v>9</v>
@@ -13269,16 +13570,16 @@
         <v>6189486656</v>
       </c>
       <c r="D496">
-        <v>3087140272</v>
+        <v>3109048832</v>
       </c>
       <c r="E496">
         <v>1331606604</v>
       </c>
       <c r="F496">
-        <v>4418746876</v>
+        <v>4440655436</v>
       </c>
       <c r="G496">
-        <v>1770739780</v>
+        <v>1748831220</v>
       </c>
       <c r="H496" t="s">
         <v>9</v>
@@ -13477,16 +13778,16 @@
         <v>7401091133</v>
       </c>
       <c r="D504">
-        <v>4673665116</v>
+        <v>4572970263</v>
       </c>
       <c r="E504">
         <v>2607739789</v>
       </c>
       <c r="F504">
-        <v>7281404905</v>
+        <v>7180710052</v>
       </c>
       <c r="G504">
-        <v>119686228</v>
+        <v>220381081</v>
       </c>
       <c r="H504" t="s">
         <v>9</v>
@@ -13529,10 +13830,10 @@
         <v>266250000</v>
       </c>
       <c r="D506">
-        <v>6838800</v>
+        <v>0</v>
       </c>
       <c r="E506">
-        <v>190238200</v>
+        <v>197077000</v>
       </c>
       <c r="F506">
         <v>197077000</v>
@@ -13763,10 +14064,10 @@
         <v>516433500</v>
       </c>
       <c r="D515">
-        <v>21491715</v>
+        <v>7568076</v>
       </c>
       <c r="E515">
-        <v>360346580</v>
+        <v>374270219</v>
       </c>
       <c r="F515">
         <v>381838295</v>
@@ -13789,16 +14090,16 @@
         <v>36180000</v>
       </c>
       <c r="D516">
-        <v>2747000</v>
+        <v>3015406</v>
       </c>
       <c r="E516">
         <v>10574568</v>
       </c>
       <c r="F516">
-        <v>13321568</v>
+        <v>13589974</v>
       </c>
       <c r="G516">
-        <v>22858432</v>
+        <v>22590026</v>
       </c>
       <c r="H516" t="s">
         <v>9</v>
@@ -13815,16 +14116,16 @@
         <v>61741000</v>
       </c>
       <c r="D517">
-        <v>0</v>
+        <v>20788000</v>
       </c>
       <c r="E517">
         <v>40855444</v>
       </c>
       <c r="F517">
-        <v>40855444</v>
+        <v>61643444</v>
       </c>
       <c r="G517">
-        <v>20885556</v>
+        <v>97556</v>
       </c>
       <c r="H517" t="s">
         <v>9</v>
@@ -13893,16 +14194,16 @@
         <v>0</v>
       </c>
       <c r="D520">
-        <v>0</v>
+        <v>25388</v>
       </c>
       <c r="E520">
         <v>748141</v>
       </c>
       <c r="F520">
-        <v>748141</v>
+        <v>773529</v>
       </c>
       <c r="G520">
-        <v>-748141</v>
+        <v>-773529</v>
       </c>
       <c r="H520" t="s">
         <v>9</v>
@@ -13919,16 +14220,16 @@
         <v>0</v>
       </c>
       <c r="D521">
-        <v>0</v>
+        <v>1800000</v>
       </c>
       <c r="E521">
         <v>115182625</v>
       </c>
       <c r="F521">
-        <v>115182625</v>
+        <v>116982625</v>
       </c>
       <c r="G521">
-        <v>-115182625</v>
+        <v>-116982625</v>
       </c>
       <c r="H521" t="s">
         <v>9</v>
@@ -13945,16 +14246,16 @@
         <v>12164281897</v>
       </c>
       <c r="D522">
-        <v>0</v>
+        <v>1068968</v>
       </c>
       <c r="E522">
         <v>8956957415</v>
       </c>
       <c r="F522">
-        <v>8956957415</v>
+        <v>8958026383</v>
       </c>
       <c r="G522">
-        <v>3207324482</v>
+        <v>3206255514</v>
       </c>
       <c r="H522" t="s">
         <v>9</v>
@@ -13997,16 +14298,16 @@
         <v>10801404197</v>
       </c>
       <c r="D524">
-        <v>0</v>
+        <v>79545016</v>
       </c>
       <c r="E524">
         <v>9796841081</v>
       </c>
       <c r="F524">
-        <v>9796841081</v>
+        <v>9876386097</v>
       </c>
       <c r="G524">
-        <v>1004563116</v>
+        <v>925018100</v>
       </c>
       <c r="H524" t="s">
         <v>9</v>
@@ -14179,16 +14480,16 @@
         <v>64019485320</v>
       </c>
       <c r="D531">
-        <v>14431488399</v>
+        <v>14396453605</v>
       </c>
       <c r="E531">
-        <v>40616310114</v>
+        <v>40686772553</v>
       </c>
       <c r="F531">
-        <v>55047798513</v>
+        <v>55083226158</v>
       </c>
       <c r="G531">
-        <v>8971686807</v>
+        <v>8936259162</v>
       </c>
       <c r="H531">
         <v>850782250</v>
@@ -14205,10 +14506,10 @@
         <v>5572131338</v>
       </c>
       <c r="D532">
-        <v>1782973068</v>
+        <v>1641723068</v>
       </c>
       <c r="E532">
-        <v>3781033270</v>
+        <v>3922283270</v>
       </c>
       <c r="F532">
         <v>5564006338</v>
@@ -14283,10 +14584,10 @@
         <v>2166235262</v>
       </c>
       <c r="D535">
-        <v>1729853601</v>
+        <v>1284417699</v>
       </c>
       <c r="E535">
-        <v>436381661</v>
+        <v>881817563</v>
       </c>
       <c r="F535">
         <v>2166235262</v>
@@ -14361,10 +14662,10 @@
         <v>11576266001</v>
       </c>
       <c r="D538">
-        <v>11246822851</v>
+        <v>7366219160</v>
       </c>
       <c r="E538">
-        <v>259825808</v>
+        <v>4140429499</v>
       </c>
       <c r="F538">
         <v>11506648659</v>
@@ -14387,16 +14688,16 @@
         <v>2103744312</v>
       </c>
       <c r="D539">
-        <v>1356681115</v>
+        <v>1036023487</v>
       </c>
       <c r="E539">
-        <v>330635136</v>
+        <v>699348736</v>
       </c>
       <c r="F539">
-        <v>1687316251</v>
+        <v>1735372223</v>
       </c>
       <c r="G539">
-        <v>416428061</v>
+        <v>368372089</v>
       </c>
       <c r="H539" t="s">
         <v>9</v>
@@ -14491,10 +14792,10 @@
         <v>1710735389</v>
       </c>
       <c r="D543">
-        <v>384000000</v>
+        <v>0</v>
       </c>
       <c r="E543">
-        <v>1326735389</v>
+        <v>1710735389</v>
       </c>
       <c r="F543">
         <v>1710735389</v>
@@ -14595,16 +14896,16 @@
         <v>1539315000</v>
       </c>
       <c r="D547">
-        <v>6343694</v>
+        <v>6712544</v>
       </c>
       <c r="E547">
         <v>933071899</v>
       </c>
       <c r="F547">
-        <v>939415593</v>
+        <v>939784443</v>
       </c>
       <c r="G547">
-        <v>599899407</v>
+        <v>599530557</v>
       </c>
       <c r="H547" t="s">
         <v>9</v>
@@ -14647,16 +14948,16 @@
         <v>532875000</v>
       </c>
       <c r="D549">
-        <v>51119621</v>
+        <v>52322721</v>
       </c>
       <c r="E549">
         <v>167536270</v>
       </c>
       <c r="F549">
-        <v>218655891</v>
+        <v>219858991</v>
       </c>
       <c r="G549">
-        <v>314219109</v>
+        <v>313016009</v>
       </c>
       <c r="H549">
         <v>177625000</v>
@@ -14728,13 +15029,13 @@
         <v>7225381</v>
       </c>
       <c r="E552">
-        <v>251095601</v>
+        <v>253789351</v>
       </c>
       <c r="F552">
-        <v>258320982</v>
+        <v>261014732</v>
       </c>
       <c r="G552">
-        <v>78481518</v>
+        <v>75787768</v>
       </c>
       <c r="H552">
         <v>112267500</v>
@@ -14806,13 +15107,13 @@
         <v>0</v>
       </c>
       <c r="E555">
-        <v>7784065393</v>
+        <v>7784118830</v>
       </c>
       <c r="F555">
-        <v>7784065393</v>
+        <v>7784118830</v>
       </c>
       <c r="G555">
-        <v>2904851473</v>
+        <v>2904798036</v>
       </c>
       <c r="H555" t="s">
         <v>9</v>
@@ -15011,16 +15312,16 @@
         <v>57848682223</v>
       </c>
       <c r="D563">
-        <v>19245745658</v>
+        <v>14075370387</v>
       </c>
       <c r="E563">
-        <v>31864701745</v>
+        <v>37087452125</v>
       </c>
       <c r="F563">
-        <v>51110447403</v>
+        <v>51162822512</v>
       </c>
       <c r="G563">
-        <v>6738234820</v>
+        <v>6685859711</v>
       </c>
       <c r="H563">
         <v>720558750</v>
@@ -15031,25 +15332,25 @@
         <v>130</v>
       </c>
       <c r="B564">
-        <v>1118540641744</v>
+        <v>1114653868055</v>
       </c>
       <c r="C564">
-        <v>1109231301920</v>
+        <v>1108157528231</v>
       </c>
       <c r="D564">
-        <v>414927051289</v>
+        <v>387069966949</v>
       </c>
       <c r="E564">
-        <v>552152652380</v>
+        <v>585636774332</v>
       </c>
       <c r="F564">
-        <v>967079703669</v>
+        <v>972706741281</v>
       </c>
       <c r="G564">
-        <v>142151598251</v>
+        <v>135450786950</v>
       </c>
       <c r="H564">
-        <v>9309339824</v>
+        <v>6496339824</v>
       </c>
     </row>
   </sheetData>

</xml_diff>